<commit_message>
feat: single 55,000 MMK lifetime plan, gemini 3.8 flash essay grader, fix mobile horizontal scroll and button wrapping
</commit_message>
<xml_diff>
--- a/IELTS_Studio_Voucher_Codes.xlsx
+++ b/IELTS_Studio_Voucher_Codes.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voucher Codes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lifetime Vouchers (55,000 MMK)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,10 +458,10 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
@@ -534,12 +534,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -549,12 +549,12 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Campaign / Testing</t>
+          <t>Campaign / Promo Launch</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Marketing Launch</t>
+          <t>Marketing Launch VIP</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -616,22 +616,22 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Myanmar Community</t>
+          <t>Myanmar Community VIP</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -698,12 +698,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>99,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1164,12 +1164,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1190,12 +1190,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1205,12 +1205,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1246,12 +1246,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1272,12 +1272,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1287,12 +1287,12 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1328,12 +1328,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1354,12 +1354,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1369,12 +1369,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1395,12 +1395,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1410,12 +1410,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1436,12 +1436,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1451,12 +1451,12 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1477,12 +1477,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1492,12 +1492,12 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1518,12 +1518,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>intensive</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>30-Day Intensive Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1533,12 +1533,12 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>30 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1559,27 +1559,27 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1600,27 +1600,27 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1641,27 +1641,27 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1682,27 +1682,27 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1723,27 +1723,27 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1764,27 +1764,27 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1805,27 +1805,27 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1846,27 +1846,27 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1887,27 +1887,27 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1928,27 +1928,27 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>sprint</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>7-Day Sprint Pass</t>
+          <t>Lifetime Studio Pass</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>25,000 MMK</t>
+          <t>55,000 MMK</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>Lifetime (Never Expires)</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Batch 1 Sales</t>
+          <t>Batch 1 Lifetime Sales</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">

</xml_diff>